<commit_message>
added saving of ADC buffer data on interrupt
</commit_message>
<xml_diff>
--- a/Hardware/Other/bar graph plan.xlsx
+++ b/Hardware/Other/bar graph plan.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/69f5ad8fb782b24f/Documents/Power Amp/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/69f5ad8fb782b24f/Documents/GitHub/Home-Audio-System/Hardware/Other/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="23" documentId="8_{6977106E-E324-46AF-97FA-091F3A60693E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{89CBB480-DDA5-4843-935B-6396629A503C}"/>
+  <xr:revisionPtr revIDLastSave="33" documentId="8_{6977106E-E324-46AF-97FA-091F3A60693E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C91BD599-1051-456D-BE90-56AEACA14EC4}"/>
   <bookViews>
-    <workbookView xWindow="345" yWindow="345" windowWidth="28800" windowHeight="15345" xr2:uid="{3A2E11FE-718E-4967-83F6-98EE0E1B199E}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{3A2E11FE-718E-4967-83F6-98EE0E1B199E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -126,10 +126,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -507,7 +503,7 @@
         <v>-3.0022346522555381</v>
       </c>
       <c r="M3">
-        <v>1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
@@ -537,7 +533,7 @@
         <v>-6.0078857519881614</v>
       </c>
       <c r="M4">
-        <v>2</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
@@ -553,7 +549,7 @@
         <v>-9.001886673395056</v>
       </c>
       <c r="M5">
-        <v>3</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
@@ -569,7 +565,7 @@
         <v>-12.007336666170348</v>
       </c>
       <c r="M6">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
@@ -588,7 +584,7 @@
         <v>-15.004571373094745</v>
       </c>
       <c r="M7">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
@@ -615,7 +611,7 @@
         <v>-17.99420492681126</v>
       </c>
       <c r="M8">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
@@ -642,7 +638,7 @@
         <v>-21.001341670225994</v>
       </c>
       <c r="M9">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
@@ -669,7 +665,7 @@
         <v>-24.014804840090882</v>
       </c>
       <c r="M10">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
@@ -696,7 +692,7 @@
         <v>-26.998177164746899</v>
       </c>
       <c r="M11">
-        <v>9</v>
+        <v>2</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
@@ -723,7 +719,7 @@
         <v>-30.035404753370507</v>
       </c>
       <c r="M12">
-        <v>10</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.25">

</xml_diff>